<commit_message>
Nang cap he thong nhan dien file thong minh va dong bo cap nhat so lieu tu may khac
</commit_message>
<xml_diff>
--- a/đầu vào/Tháng 8/TK 336 - HCM.xlsx
+++ b/đầu vào/Tháng 8/TK 336 - HCM.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. TCKT_PCVT\5.Tổng hợp\T8\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngamvp\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66888512-96D9-4EAD-BAD2-BCE5531858BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{20D2D462-4D9B-40AA-BDF2-16BE78E9A067}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8076"/>
   </bookViews>
   <sheets>
-    <sheet name="EVN_GL_094___Sổ_chi_tiết_t_1009" sheetId="2" r:id="rId1"/>
+    <sheet name="EVN_GL_094___Sổ_chi_tiết_t_1109" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -135,7 +135,7 @@
     <t>29 308 679</t>
   </si>
   <si>
-    <t>Draft</t>
+    <t>Final post to GL</t>
   </si>
   <si>
     <t xml:space="preserve">NHIHY.HCM.NG </t>
@@ -784,7 +784,7 @@
     <t>(Ký, họ tên, đóng dấu)</t>
   </si>
   <si>
-    <t>EVN_GL_094, người in: NGAMVP.HCM.NG, ngày in: 10/09/2026 09:06:56</t>
+    <t>EVN_GL_094, người in: NGAMVP.HCM.NG, ngày in: 11/09/2026 14:24:29</t>
   </si>
   <si>
     <t>Trang 1/1</t>
@@ -793,7 +793,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1438,6 +1438,15 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1480,6 +1489,39 @@
     <xf numFmtId="0" fontId="20" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -1489,56 +1531,14 @@
     <xf numFmtId="0" fontId="23" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1599,9 +1599,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1639,7 +1639,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1745,7 +1745,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1887,14 +1887,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1904,7 +1904,7 @@
     <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1912,19 +1912,19 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="4"/>
     </row>
     <row r="2" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="26"/>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="26"/>
+      <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1933,1201 +1933,1273 @@
       <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
+      <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="28"/>
+      <c r="B6" s="6"/>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="6"/>
     </row>
     <row r="9" spans="1:9" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="29" t="s">
+      <c r="C9" s="23"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="22"/>
+      <c r="B10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="5" t="s">
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="36"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
     </row>
     <row r="12" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10" t="s">
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="11"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="14"/>
     </row>
     <row r="13" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="16">
         <v>46265</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="19">
         <v>9115</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="17" t="s">
+      <c r="F13" s="17"/>
+      <c r="G13" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="15" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="10" t="s">
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="H14" s="9"/>
-      <c r="I14" s="11"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="14"/>
     </row>
     <row r="15" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="10" t="s">
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="11"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="14"/>
     </row>
     <row r="16" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="36"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="28"/>
     </row>
     <row r="17" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="11"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="14"/>
     </row>
     <row r="18" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="13">
+      <c r="A18" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="16">
         <v>46237</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="17" t="s">
+      <c r="D18" s="19">
+        <v>9193</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="17"/>
+      <c r="G18" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I18" s="12" t="s">
+      <c r="H18" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="13">
+      <c r="A19" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="16">
         <v>46237</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="17" t="s">
+      <c r="D19" s="19">
+        <v>9193</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="17"/>
+      <c r="G19" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="H19" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I19" s="12" t="s">
+      <c r="H19" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I19" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="13">
+      <c r="A20" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="16">
         <v>46238</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" s="14"/>
-      <c r="G20" s="17" t="s">
+      <c r="D20" s="19">
+        <v>9167</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="17"/>
+      <c r="G20" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="H20" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I20" s="12" t="s">
+      <c r="H20" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="13">
+      <c r="A21" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="16">
         <v>46239</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="14"/>
-      <c r="E21" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="17" t="s">
+      <c r="D21" s="19">
+        <v>9191</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="17"/>
+      <c r="G21" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="H21" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I21" s="12" t="s">
+      <c r="H21" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I21" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="13">
+      <c r="A22" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="16">
         <v>46240</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="17" t="s">
+      <c r="D22" s="19">
+        <v>9171</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="17"/>
+      <c r="G22" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="H22" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I22" s="12" t="s">
+      <c r="H22" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I22" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="13">
+      <c r="A23" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="16">
         <v>46240</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="17" t="s">
+      <c r="D23" s="19">
+        <v>9171</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="17"/>
+      <c r="G23" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="H23" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I23" s="12" t="s">
+      <c r="H23" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I23" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="13">
+      <c r="A24" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="16">
         <v>46241</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="17" t="s">
+      <c r="D24" s="19">
+        <v>9192</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="17"/>
+      <c r="G24" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="H24" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I24" s="12" t="s">
+      <c r="H24" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="13">
+      <c r="A25" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="16">
         <v>46244</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="17" t="s">
+      <c r="D25" s="19">
+        <v>9169</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" s="17"/>
+      <c r="G25" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="H25" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I25" s="12" t="s">
+      <c r="H25" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I25" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="13">
+      <c r="A26" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="16">
         <v>46244</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F26" s="14"/>
-      <c r="G26" s="17" t="s">
+      <c r="D26" s="19">
+        <v>9169</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="17"/>
+      <c r="G26" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="H26" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I26" s="12" t="s">
+      <c r="H26" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I26" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="13">
+      <c r="A27" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="16">
         <v>46244</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="C27" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="17" t="s">
+      <c r="D27" s="19">
+        <v>9169</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="17"/>
+      <c r="G27" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="H27" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I27" s="12" t="s">
+      <c r="H27" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="13">
+      <c r="A28" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="16">
         <v>46245</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" s="14"/>
-      <c r="G28" s="17" t="s">
+      <c r="D28" s="19">
+        <v>9183</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="17"/>
+      <c r="G28" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="H28" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I28" s="12" t="s">
+      <c r="H28" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I28" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="13">
+      <c r="A29" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="16">
         <v>46246</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F29" s="14"/>
-      <c r="G29" s="17" t="s">
+      <c r="D29" s="19">
+        <v>9194</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="17"/>
+      <c r="G29" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="H29" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I29" s="12" t="s">
+      <c r="H29" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="13">
+      <c r="A30" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="16">
         <v>46246</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" s="14"/>
-      <c r="G30" s="17" t="s">
+      <c r="D30" s="19">
+        <v>9194</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="17"/>
+      <c r="G30" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H30" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I30" s="12" t="s">
+      <c r="H30" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I30" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="13">
+      <c r="A31" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="16">
         <v>46247</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F31" s="14"/>
-      <c r="G31" s="17" t="s">
+      <c r="D31" s="19">
+        <v>9166</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F31" s="17"/>
+      <c r="G31" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="H31" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I31" s="12" t="s">
+      <c r="H31" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I31" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="13">
+      <c r="A32" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="16">
         <v>46248</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D32" s="14"/>
-      <c r="E32" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F32" s="14"/>
-      <c r="G32" s="17" t="s">
+      <c r="D32" s="19">
+        <v>9188</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F32" s="17"/>
+      <c r="G32" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="H32" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I32" s="12" t="s">
+      <c r="H32" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I32" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B33" s="13">
+      <c r="A33" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="16">
         <v>46248</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F33" s="14"/>
-      <c r="G33" s="17" t="s">
+      <c r="D33" s="19">
+        <v>9188</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F33" s="17"/>
+      <c r="G33" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H33" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I33" s="12" t="s">
+      <c r="H33" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I33" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" s="13">
+      <c r="A34" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="16">
         <v>46248</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F34" s="14"/>
-      <c r="G34" s="17" t="s">
+      <c r="D34" s="19">
+        <v>9188</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F34" s="17"/>
+      <c r="G34" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="H34" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I34" s="12" t="s">
+      <c r="H34" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I34" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="13">
+      <c r="A35" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="16">
         <v>46251</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F35" s="14"/>
-      <c r="G35" s="17" t="s">
+      <c r="D35" s="19">
+        <v>9185</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F35" s="17"/>
+      <c r="G35" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="H35" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I35" s="12" t="s">
+      <c r="H35" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I35" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" s="13">
+      <c r="A36" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="16">
         <v>46251</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F36" s="14"/>
-      <c r="G36" s="17" t="s">
+      <c r="D36" s="19">
+        <v>9185</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="17"/>
+      <c r="G36" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="H36" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I36" s="12" t="s">
+      <c r="H36" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I36" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B37" s="13">
+      <c r="A37" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" s="16">
         <v>46251</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D37" s="14"/>
-      <c r="E37" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F37" s="14"/>
-      <c r="G37" s="17" t="s">
+      <c r="D37" s="19">
+        <v>9185</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F37" s="17"/>
+      <c r="G37" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="H37" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I37" s="12" t="s">
+      <c r="H37" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I37" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" s="13">
+      <c r="A38" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="16">
         <v>46251</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="D38" s="14"/>
-      <c r="E38" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F38" s="14"/>
-      <c r="G38" s="17" t="s">
+      <c r="D38" s="19">
+        <v>9185</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F38" s="17"/>
+      <c r="G38" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="H38" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I38" s="12" t="s">
+      <c r="H38" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" s="13">
+      <c r="A39" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B39" s="16">
         <v>46252</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D39" s="14"/>
-      <c r="E39" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F39" s="14"/>
-      <c r="G39" s="17" t="s">
+      <c r="D39" s="19">
+        <v>9165</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F39" s="17"/>
+      <c r="G39" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I39" s="12" t="s">
+      <c r="H39" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="13">
+      <c r="A40" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" s="16">
         <v>46253</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C40" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D40" s="14"/>
-      <c r="E40" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F40" s="14"/>
-      <c r="G40" s="17" t="s">
+      <c r="D40" s="19">
+        <v>9173</v>
+      </c>
+      <c r="E40" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F40" s="17"/>
+      <c r="G40" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="H40" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I40" s="12" t="s">
+      <c r="H40" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I40" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41" s="13">
+      <c r="A41" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="16">
         <v>46253</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D41" s="14"/>
-      <c r="E41" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F41" s="14"/>
-      <c r="G41" s="17" t="s">
+      <c r="D41" s="19">
+        <v>9173</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F41" s="17"/>
+      <c r="G41" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="H41" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I41" s="12" t="s">
+      <c r="H41" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I41" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B42" s="13">
+      <c r="A42" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="16">
         <v>46254</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="C42" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D42" s="14"/>
-      <c r="E42" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F42" s="14"/>
-      <c r="G42" s="17" t="s">
+      <c r="D42" s="19">
+        <v>9180</v>
+      </c>
+      <c r="E42" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F42" s="17"/>
+      <c r="G42" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="H42" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I42" s="12" t="s">
+      <c r="H42" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I42" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B43" s="13">
+      <c r="A43" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="16">
         <v>46255</v>
       </c>
-      <c r="C43" s="15" t="s">
+      <c r="C43" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="D43" s="14"/>
-      <c r="E43" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F43" s="14"/>
-      <c r="G43" s="17" t="s">
+      <c r="D43" s="19">
+        <v>9174</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F43" s="17"/>
+      <c r="G43" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="H43" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I43" s="12" t="s">
+      <c r="H43" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I43" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B44" s="13">
+      <c r="A44" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" s="16">
         <v>46256</v>
       </c>
-      <c r="C44" s="15" t="s">
+      <c r="C44" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D44" s="14"/>
-      <c r="E44" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F44" s="14"/>
-      <c r="G44" s="17" t="s">
+      <c r="D44" s="19">
+        <v>9190</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F44" s="17"/>
+      <c r="G44" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="H44" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I44" s="12" t="s">
+      <c r="H44" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I44" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" s="13">
+      <c r="A45" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B45" s="16">
         <v>46258</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="C45" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D45" s="14"/>
-      <c r="E45" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F45" s="14"/>
-      <c r="G45" s="17" t="s">
+      <c r="D45" s="19">
+        <v>9175</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F45" s="17"/>
+      <c r="G45" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="H45" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I45" s="12" t="s">
+      <c r="H45" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I45" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" s="13">
+      <c r="A46" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B46" s="16">
         <v>46258</v>
       </c>
-      <c r="C46" s="15" t="s">
+      <c r="C46" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D46" s="14"/>
-      <c r="E46" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F46" s="14"/>
-      <c r="G46" s="17" t="s">
+      <c r="D46" s="19">
+        <v>9175</v>
+      </c>
+      <c r="E46" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F46" s="17"/>
+      <c r="G46" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="H46" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I46" s="12" t="s">
+      <c r="H46" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I46" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B47" s="13">
+      <c r="A47" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B47" s="16">
         <v>46259</v>
       </c>
-      <c r="C47" s="15" t="s">
+      <c r="C47" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="D47" s="14"/>
-      <c r="E47" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F47" s="14"/>
-      <c r="G47" s="17" t="s">
+      <c r="D47" s="19">
+        <v>9177</v>
+      </c>
+      <c r="E47" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F47" s="17"/>
+      <c r="G47" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="H47" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I47" s="12" t="s">
+      <c r="H47" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I47" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B48" s="13">
+      <c r="A48" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="16">
         <v>46260</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C48" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D48" s="14"/>
-      <c r="E48" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F48" s="14"/>
-      <c r="G48" s="17" t="s">
+      <c r="D48" s="19">
+        <v>9168</v>
+      </c>
+      <c r="E48" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" s="17"/>
+      <c r="G48" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="H48" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I48" s="12" t="s">
+      <c r="H48" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I48" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B49" s="13">
+      <c r="A49" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B49" s="16">
         <v>46260</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="C49" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="D49" s="14"/>
-      <c r="E49" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F49" s="14"/>
-      <c r="G49" s="17" t="s">
+      <c r="D49" s="19">
+        <v>9168</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" s="17"/>
+      <c r="G49" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H49" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I49" s="12" t="s">
+      <c r="H49" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I49" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B50" s="13">
+      <c r="A50" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" s="16">
         <v>46260</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="C50" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="D50" s="14"/>
-      <c r="E50" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F50" s="14"/>
-      <c r="G50" s="17" t="s">
+      <c r="D50" s="19">
+        <v>9168</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F50" s="17"/>
+      <c r="G50" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="H50" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I50" s="12" t="s">
+      <c r="H50" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I50" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B51" s="13">
+      <c r="A51" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B51" s="16">
         <v>46261</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="C51" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="D51" s="14"/>
-      <c r="E51" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F51" s="14"/>
-      <c r="G51" s="17" t="s">
+      <c r="D51" s="19">
+        <v>9176</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F51" s="17"/>
+      <c r="G51" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="H51" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I51" s="12" t="s">
+      <c r="H51" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I51" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B52" s="13">
+      <c r="A52" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B52" s="16">
         <v>46262</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="C52" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="14"/>
-      <c r="E52" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F52" s="14"/>
-      <c r="G52" s="17" t="s">
+      <c r="D52" s="19">
+        <v>9186</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F52" s="17"/>
+      <c r="G52" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H52" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I52" s="12" t="s">
+      <c r="H52" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I52" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B53" s="13">
+      <c r="A53" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B53" s="16">
         <v>46262</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C53" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="D53" s="14"/>
-      <c r="E53" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F53" s="14"/>
-      <c r="G53" s="17" t="s">
+      <c r="D53" s="19">
+        <v>9186</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F53" s="17"/>
+      <c r="G53" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="H53" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="I53" s="12" t="s">
+      <c r="H53" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I53" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="13">
+      <c r="B54" s="16">
         <v>46265</v>
       </c>
-      <c r="C54" s="15" t="s">
+      <c r="C54" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D54" s="16">
+      <c r="D54" s="19">
         <v>9097</v>
       </c>
-      <c r="E54" s="16" t="s">
+      <c r="E54" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="F54" s="17" t="s">
+      <c r="F54" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="G54" s="14"/>
-      <c r="H54" s="16" t="s">
+      <c r="G54" s="17"/>
+      <c r="H54" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="I54" s="12" t="s">
+      <c r="I54" s="15" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B55" s="13">
+      <c r="B55" s="16">
         <v>46265</v>
       </c>
-      <c r="C55" s="15" t="s">
+      <c r="C55" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D55" s="16">
+      <c r="D55" s="19">
         <v>9097</v>
       </c>
-      <c r="E55" s="16" t="s">
+      <c r="E55" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="F55" s="17" t="s">
+      <c r="F55" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="G55" s="14"/>
-      <c r="H55" s="16" t="s">
+      <c r="G55" s="17"/>
+      <c r="H55" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="I55" s="12" t="s">
+      <c r="I55" s="15" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="23" t="s">
+      <c r="A56" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B56" s="24"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="10" t="s">
+      <c r="B56" s="30"/>
+      <c r="C56" s="30"/>
+      <c r="D56" s="30"/>
+      <c r="E56" s="31"/>
+      <c r="F56" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G56" s="10" t="s">
+      <c r="G56" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="H56" s="9"/>
-      <c r="I56" s="11"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="14"/>
     </row>
     <row r="57" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="23" t="s">
+      <c r="A57" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="24"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="11"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+      <c r="D57" s="30"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="14"/>
     </row>
     <row r="58" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="18" t="s">
+      <c r="A58" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B58" s="9"/>
-      <c r="C58" s="10" t="s">
+      <c r="B58" s="12"/>
+      <c r="C58" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
     </row>
     <row r="59" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="C59" s="10" t="s">
+      <c r="C59" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
     </row>
     <row r="60" spans="1:9" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="18" t="s">
+      <c r="A60" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="B60" s="9"/>
-      <c r="C60" s="10" t="s">
+      <c r="B60" s="12"/>
+      <c r="C60" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
     </row>
     <row r="61" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="37"/>
-      <c r="B61" s="37"/>
-      <c r="C61" s="19" t="s">
+      <c r="A61" s="35"/>
+      <c r="B61" s="35"/>
+      <c r="C61" s="33" t="s">
         <v>117</v>
       </c>
     </row>
@@ -3141,28 +3213,24 @@
       </c>
     </row>
     <row r="63" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="20" t="s">
+      <c r="A63" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="B63" s="8"/>
-      <c r="C63" s="20" t="s">
+      <c r="B63" s="11"/>
+      <c r="C63" s="34" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="12.15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="21" t="s">
+      <c r="A65" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="B65" s="22" t="s">
+      <c r="B65" s="37" t="s">
         <v>123</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="A11:I11"/>
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A15:E15"/>
@@ -3170,6 +3238,11 @@
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A57:E57"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="A11:I11"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="B1:B3"/>
     <mergeCell ref="A5:B5"/>
@@ -3177,7 +3250,6 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E9:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>